<commit_message>
checkpoint before checking out master
</commit_message>
<xml_diff>
--- a/Fichas/Ficha.xlsx
+++ b/Fichas/Ficha.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PDE\DEMO\Fichas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65020EAA-7050-4D84-87C5-C34293A406BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50A21E7D-D056-4190-B062-DBAA989173F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PI FALTA DE FRANCOBORDO" sheetId="1" r:id="rId1"/>
@@ -41,9 +41,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
-    <t>MODELO DE  CÁLCULO</t>
-  </si>
-  <si>
     <t>Input del modelo</t>
   </si>
   <si>
@@ -54,9 +51,6 @@
   </si>
   <si>
     <t>Vulnerabilidad</t>
-  </si>
-  <si>
-    <t>MODELO ECONÓMICO</t>
   </si>
   <si>
     <t>Driver</t>
@@ -118,6 +112,33 @@
   </si>
   <si>
     <t>Número de horas al año en las que el francobordo disponible del muelle es inferior al francobordo mínimo operativo.</t>
+  </si>
+  <si>
+    <t>Especificar: p.e Régimen y si alguna variables es a pie de dique o muelle etc</t>
+  </si>
+  <si>
+    <t>Revisar y corregir todo lo que esté en rojo</t>
+  </si>
+  <si>
+    <t>TWL= MA + MM + SLR + Sobreelevación hidráulica + Nivel Precipitación</t>
+  </si>
+  <si>
+    <t>Francobordo mínimo operativo.</t>
+  </si>
+  <si>
+    <t>Reducción de francobordo por TWL</t>
+  </si>
+  <si>
+    <t>PI (ELO): PERDIDA D EINGRESO POR INTERRUPCIÓN OPERATIVA DEBIDO A LA FALTA DE FRANCOBORDO MÍNIMO OPERATIVO</t>
+  </si>
+  <si>
+    <t>Pérdida de ingreso por interrpución operativa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Para cada escenario futuro se compara el número de horas de inoperatividad con el periodo histórico. Si la inoperatividad disminuye o se mantiene, la pérdida de ingresos se considera nula. Si aumenta, la pérdida se calcula multiplicando el incremento de horas no operativas por el ingreso horario medio de la terminal. </t>
+  </si>
+  <si>
+    <t>Tasas portuarias efectivamente reguladas y los cánones concesionales.</t>
   </si>
   <si>
     <r>
@@ -170,17 +191,6 @@
     </r>
     <r>
       <rPr>
-        <b/>
-        <vertAlign val="superscript"/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>1</t>
-    </r>
-    <r>
-      <rPr>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
@@ -190,38 +200,17 @@
     </r>
   </si>
   <si>
-    <t>Especificar: p.e Régimen y si alguna variables es a pie de dique o muelle etc</t>
-  </si>
-  <si>
-    <t>Revisar y corregir todo lo que esté en rojo</t>
-  </si>
-  <si>
-    <t>TWL= MA + MM + SLR + Sobreelevación hidráulica + Nivel Precipitación</t>
-  </si>
-  <si>
-    <t>Francobordo mínimo operativo.</t>
-  </si>
-  <si>
-    <t>Reducción de francobordo por TWL</t>
-  </si>
-  <si>
-    <t>PI (ELO): PERDIDA D EINGRESO POR INTERRUPCIÓN OPERATIVA DEBIDO A LA FALTA DE FRANCOBORDO MÍNIMO OPERATIVO</t>
-  </si>
-  <si>
-    <t>Pérdida de ingreso por interrpución operativa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Para cada escenario futuro se compara el número de horas de inoperatividad con el periodo histórico. Si la inoperatividad disminuye o se mantiene, la pérdida de ingresos se considera nula. Si aumenta, la pérdida se calcula multiplicando el incremento de horas no operativas por el ingreso horario medio de la terminal. </t>
-  </si>
-  <si>
-    <t>Tasas portuarias efectivamente reguladas y los cánones concesionales.</t>
+    <t xml:space="preserve">MODELO DE IMPACTO FÍSICO </t>
+  </si>
+  <si>
+    <t>MODELO DE IMPACTO ECONOMICO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -276,14 +265,6 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <b/>
-      <vertAlign val="superscript"/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -419,6 +400,32 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -432,32 +439,6 @@
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -489,8 +470,8 @@
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>1713163</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>25244</xdr:rowOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>53819</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -531,8 +512,8 @@
       <xdr:rowOff>176212</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3800207" cy="549831"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="CuadroTexto 6">
@@ -605,7 +586,7 @@
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
                             <a:effectLst/>
-                            <a:latin typeface="+mn-lt"/>
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                             <a:ea typeface="+mn-ea"/>
                             <a:cs typeface="+mn-cs"/>
                           </a:rPr>
@@ -618,7 +599,7 @@
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
                             <a:effectLst/>
-                            <a:latin typeface="+mn-lt"/>
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                             <a:ea typeface="+mn-ea"/>
                             <a:cs typeface="+mn-cs"/>
                           </a:rPr>
@@ -630,7 +611,7 @@
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
                             <a:effectLst/>
-                            <a:latin typeface="+mn-lt"/>
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                             <a:ea typeface="+mn-ea"/>
                             <a:cs typeface="+mn-cs"/>
                           </a:rPr>
@@ -644,7 +625,7 @@
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
                             <a:effectLst/>
-                            <a:latin typeface="+mn-lt"/>
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                             <a:ea typeface="+mn-ea"/>
                             <a:cs typeface="+mn-cs"/>
                           </a:rPr>
@@ -658,7 +639,7 @@
                           <a:schemeClr val="tx1"/>
                         </a:solidFill>
                         <a:effectLst/>
-                        <a:latin typeface="+mn-lt"/>
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                         <a:ea typeface="+mn-ea"/>
                         <a:cs typeface="+mn-cs"/>
                       </a:rPr>
@@ -672,7 +653,7 @@
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
                             <a:effectLst/>
-                            <a:latin typeface="+mn-lt"/>
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                             <a:ea typeface="+mn-ea"/>
                             <a:cs typeface="+mn-cs"/>
                           </a:rPr>
@@ -685,7 +666,7 @@
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
                             <a:effectLst/>
-                            <a:latin typeface="+mn-lt"/>
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                             <a:ea typeface="+mn-ea"/>
                             <a:cs typeface="+mn-cs"/>
                           </a:rPr>
@@ -703,7 +684,7 @@
                                   <a:schemeClr val="tx1"/>
                                 </a:solidFill>
                                 <a:effectLst/>
-                                <a:latin typeface="+mn-lt"/>
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                 <a:ea typeface="+mn-ea"/>
                                 <a:cs typeface="+mn-cs"/>
                               </a:rPr>
@@ -716,7 +697,7 @@
                                   <a:schemeClr val="tx1"/>
                                 </a:solidFill>
                                 <a:effectLst/>
-                                <a:latin typeface="+mn-lt"/>
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                 <a:ea typeface="+mn-ea"/>
                                 <a:cs typeface="+mn-cs"/>
                               </a:rPr>
@@ -728,7 +709,7 @@
                                   <a:schemeClr val="tx1"/>
                                 </a:solidFill>
                                 <a:effectLst/>
-                                <a:latin typeface="+mn-lt"/>
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                 <a:ea typeface="+mn-ea"/>
                                 <a:cs typeface="+mn-cs"/>
                               </a:rPr>
@@ -742,7 +723,7 @@
                                       <a:schemeClr val="tx1"/>
                                     </a:solidFill>
                                     <a:effectLst/>
-                                    <a:latin typeface="+mn-lt"/>
+                                    <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                     <a:ea typeface="+mn-ea"/>
                                     <a:cs typeface="+mn-cs"/>
                                   </a:rPr>
@@ -757,7 +738,7 @@
                                           <a:schemeClr val="tx1"/>
                                         </a:solidFill>
                                         <a:effectLst/>
-                                        <a:latin typeface="+mn-lt"/>
+                                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                         <a:ea typeface="+mn-ea"/>
                                         <a:cs typeface="+mn-cs"/>
                                       </a:rPr>
@@ -770,7 +751,7 @@
                                           <a:schemeClr val="tx1"/>
                                         </a:solidFill>
                                         <a:effectLst/>
-                                        <a:latin typeface="+mn-lt"/>
+                                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                         <a:ea typeface="+mn-ea"/>
                                         <a:cs typeface="+mn-cs"/>
                                       </a:rPr>
@@ -784,7 +765,7 @@
                                           <a:schemeClr val="tx1"/>
                                         </a:solidFill>
                                         <a:effectLst/>
-                                        <a:latin typeface="+mn-lt"/>
+                                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                         <a:ea typeface="+mn-ea"/>
                                         <a:cs typeface="+mn-cs"/>
                                       </a:rPr>
@@ -798,7 +779,7 @@
                                       <a:schemeClr val="tx1"/>
                                     </a:solidFill>
                                     <a:effectLst/>
-                                    <a:latin typeface="+mn-lt"/>
+                                    <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                     <a:ea typeface="+mn-ea"/>
                                     <a:cs typeface="+mn-cs"/>
                                   </a:rPr>
@@ -812,7 +793,7 @@
                                           <a:schemeClr val="tx1"/>
                                         </a:solidFill>
                                         <a:effectLst/>
-                                        <a:latin typeface="+mn-lt"/>
+                                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                         <a:ea typeface="+mn-ea"/>
                                         <a:cs typeface="+mn-cs"/>
                                       </a:rPr>
@@ -825,7 +806,7 @@
                                           <a:schemeClr val="tx1"/>
                                         </a:solidFill>
                                         <a:effectLst/>
-                                        <a:latin typeface="+mn-lt"/>
+                                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                         <a:ea typeface="+mn-ea"/>
                                         <a:cs typeface="+mn-cs"/>
                                       </a:rPr>
@@ -839,7 +820,7 @@
                                           <a:schemeClr val="tx1"/>
                                         </a:solidFill>
                                         <a:effectLst/>
-                                        <a:latin typeface="+mn-lt"/>
+                                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                         <a:ea typeface="+mn-ea"/>
                                         <a:cs typeface="+mn-cs"/>
                                       </a:rPr>
@@ -851,7 +832,7 @@
                                           <a:schemeClr val="tx1"/>
                                         </a:solidFill>
                                         <a:effectLst/>
-                                        <a:latin typeface="+mn-lt"/>
+                                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                         <a:ea typeface="+mn-ea"/>
                                         <a:cs typeface="+mn-cs"/>
                                       </a:rPr>
@@ -867,7 +848,7 @@
                                       <a:schemeClr val="tx1"/>
                                     </a:solidFill>
                                     <a:effectLst/>
-                                    <a:latin typeface="+mn-lt"/>
+                                    <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                     <a:ea typeface="+mn-ea"/>
                                     <a:cs typeface="+mn-cs"/>
                                   </a:rPr>
@@ -879,7 +860,7 @@
                                       <a:schemeClr val="tx1"/>
                                     </a:solidFill>
                                     <a:effectLst/>
-                                    <a:latin typeface="+mn-lt"/>
+                                    <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                     <a:ea typeface="+mn-ea"/>
                                     <a:cs typeface="+mn-cs"/>
                                   </a:rPr>
@@ -891,7 +872,7 @@
                                       <a:schemeClr val="tx1"/>
                                     </a:solidFill>
                                     <a:effectLst/>
-                                    <a:latin typeface="+mn-lt"/>
+                                    <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                     <a:ea typeface="+mn-ea"/>
                                     <a:cs typeface="+mn-cs"/>
                                   </a:rPr>
@@ -905,7 +886,7 @@
                                   <a:schemeClr val="tx1"/>
                                 </a:solidFill>
                                 <a:effectLst/>
-                                <a:latin typeface="+mn-lt"/>
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                 <a:ea typeface="+mn-ea"/>
                                 <a:cs typeface="+mn-cs"/>
                               </a:rPr>
@@ -919,7 +900,7 @@
                                       <a:schemeClr val="tx1"/>
                                     </a:solidFill>
                                     <a:effectLst/>
-                                    <a:latin typeface="+mn-lt"/>
+                                    <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                     <a:ea typeface="+mn-ea"/>
                                     <a:cs typeface="+mn-cs"/>
                                   </a:rPr>
@@ -932,7 +913,7 @@
                                       <a:schemeClr val="tx1"/>
                                     </a:solidFill>
                                     <a:effectLst/>
-                                    <a:latin typeface="+mn-lt"/>
+                                    <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                     <a:ea typeface="+mn-ea"/>
                                     <a:cs typeface="+mn-cs"/>
                                   </a:rPr>
@@ -944,7 +925,7 @@
                                       <a:schemeClr val="tx1"/>
                                     </a:solidFill>
                                     <a:effectLst/>
-                                    <a:latin typeface="+mn-lt"/>
+                                    <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                     <a:ea typeface="+mn-ea"/>
                                     <a:cs typeface="+mn-cs"/>
                                   </a:rPr>
@@ -956,7 +937,7 @@
                                       <a:schemeClr val="tx1"/>
                                     </a:solidFill>
                                     <a:effectLst/>
-                                    <a:latin typeface="+mn-lt"/>
+                                    <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                     <a:ea typeface="+mn-ea"/>
                                     <a:cs typeface="+mn-cs"/>
                                   </a:rPr>
@@ -968,7 +949,7 @@
                                       <a:schemeClr val="tx1"/>
                                     </a:solidFill>
                                     <a:effectLst/>
-                                    <a:latin typeface="+mn-lt"/>
+                                    <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                     <a:ea typeface="+mn-ea"/>
                                     <a:cs typeface="+mn-cs"/>
                                   </a:rPr>
@@ -986,7 +967,7 @@
                           <a:schemeClr val="tx1"/>
                         </a:solidFill>
                         <a:effectLst/>
-                        <a:latin typeface="+mn-lt"/>
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                         <a:ea typeface="+mn-ea"/>
                         <a:cs typeface="+mn-cs"/>
                       </a:rPr>
@@ -1011,7 +992,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="CuadroTexto 6">
@@ -1421,151 +1402,151 @@
     <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="75.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="79.85546875" style="15"/>
+    <col min="4" max="4" width="79.85546875" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="7"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="7"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+    </row>
+    <row r="5" spans="1:3" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="15"/>
+    </row>
+    <row r="6" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="11"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="11"/>
+      <c r="B8" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="11"/>
+      <c r="B9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="12"/>
+      <c r="B10" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+    </row>
+    <row r="12" spans="1:3" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-    </row>
-    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="15"/>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-    </row>
-    <row r="5" spans="1:3" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+    </row>
+    <row r="13" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="11"/>
+      <c r="B13" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="11"/>
+      <c r="B14" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="11"/>
+      <c r="B15" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="5"/>
-    </row>
-    <row r="6" spans="1:3" ht="48" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
-      <c r="B8" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
-      <c r="B9" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="13"/>
-      <c r="B10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-    </row>
-    <row r="12" spans="1:3" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="12" t="s">
+    </row>
+    <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="11"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+    </row>
+    <row r="17" spans="1:3" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="11"/>
+      <c r="B17" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="30" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="8"/>
-      <c r="B13" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="8"/>
-      <c r="B14" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="8"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-    </row>
-    <row r="17" spans="1:3" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="8"/>
-      <c r="B17" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
     <row r="18" spans="1:3" ht="59.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="17"/>
+      <c r="A18" s="12"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="9"/>
     </row>
     <row r="19" spans="1:3" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="15"/>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
+      <c r="A19" s="7"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>